<commit_message>
feat: complete end-to-end multi-agent verification, ISO/IATF reporting, and cloud deployment configuration
</commit_message>
<xml_diff>
--- a/backend/data/inspection/measurements.xlsx
+++ b/backend/data/inspection/measurements.xlsx
@@ -5605,7 +5605,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>49.996</v>
+        <v>49.999</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -5646,7 +5646,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>50.004</v>
+        <v>50.005</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>50.008</v>
+        <v>50.013</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -5728,7 +5728,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>50.022</v>
+        <v>50.009</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -5769,7 +5769,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>50.021</v>
+        <v>50.022</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -5810,7 +5810,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>50.03</v>
+        <v>50.026</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -5851,7 +5851,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>50.023</v>
+        <v>50.032</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -5933,7 +5933,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>50.044</v>
+        <v>50.052</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -5950,11 +5950,11 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>conforming</t>
+          <t>nonconforming</t>
         </is>
       </c>
       <c r="I135" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="136">
@@ -5974,7 +5974,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>50.045</v>
+        <v>50.042</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>50.055</v>
+        <v>50.047</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -6032,11 +6032,11 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I137" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -6097,7 +6097,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>50.067</v>
+        <v>50.057</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -6118,7 +6118,7 @@
         </is>
       </c>
       <c r="I139" t="n">
-        <v>0.017</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="140">
@@ -6138,7 +6138,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>50.076</v>
+        <v>50.062</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -6159,7 +6159,7 @@
         </is>
       </c>
       <c r="I140" t="n">
-        <v>0.026</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="141">
@@ -6179,7 +6179,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>50.068</v>
+        <v>50.076</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -6200,7 +6200,7 @@
         </is>
       </c>
       <c r="I141" t="n">
-        <v>0.018</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="142">
@@ -6220,7 +6220,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>85.01000000000001</v>
+        <v>85.026</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -6261,7 +6261,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>85.026</v>
+        <v>84.985</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -6302,7 +6302,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>85.008</v>
+        <v>84.979</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -6343,7 +6343,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>84.995</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -6384,7 +6384,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>85.008</v>
+        <v>84.999</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -6425,7 +6425,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>85.01600000000001</v>
+        <v>85.003</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -6466,7 +6466,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85.011</v>
+        <v>84.997</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -6507,7 +6507,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>85.00700000000001</v>
+        <v>85.005</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -6548,7 +6548,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>85.015</v>
+        <v>84.982</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -6589,7 +6589,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>85.01600000000001</v>
+        <v>85.02</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -6630,7 +6630,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>85.01900000000001</v>
+        <v>84.999</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -6671,7 +6671,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>85.009</v>
+        <v>85.01600000000001</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>84.998</v>
+        <v>85.005</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -6753,7 +6753,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>85.002</v>
+        <v>85.006</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -6794,7 +6794,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>85.017</v>
+        <v>85.008</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -6835,7 +6835,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>12.506</v>
+        <v>12.493</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -6876,7 +6876,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>12.509</v>
+        <v>12.522</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -6917,7 +6917,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>12.519</v>
+        <v>12.483</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -6958,7 +6958,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>12.503</v>
+        <v>12.479</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -6999,7 +6999,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>12.51</v>
+        <v>12.503</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -7040,7 +7040,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>12.499</v>
+        <v>12.515</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>12.52</v>
+        <v>12.524</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -7122,7 +7122,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>12.491</v>
+        <v>12.494</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -7163,7 +7163,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>12.525</v>
+        <v>12.515</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -7245,7 +7245,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>12.48</v>
+        <v>12.498</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -7286,7 +7286,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>12.502</v>
+        <v>12.512</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -7327,7 +7327,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>12.49</v>
+        <v>12.509</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -7368,7 +7368,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>12.512</v>
+        <v>12.478</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -7409,7 +7409,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>12.491</v>
+        <v>12.521</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -7450,7 +7450,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>49.993</v>
+        <v>50.023</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -7491,7 +7491,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>50.022</v>
+        <v>49.984</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -7532,7 +7532,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>49.983</v>
+        <v>50.004</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>49.979</v>
+        <v>49.989</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -7614,7 +7614,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>50.003</v>
+        <v>49.999</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -7655,7 +7655,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>50.015</v>
+        <v>50.005</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -7696,7 +7696,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>50.024</v>
+        <v>50.004</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>49.994</v>
+        <v>50.006</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -7778,7 +7778,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>50.015</v>
+        <v>50.023</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -7819,7 +7819,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>49.999</v>
+        <v>50.006</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -7860,7 +7860,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>49.998</v>
+        <v>49.997</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -7901,7 +7901,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>50.012</v>
+        <v>50.013</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -7942,7 +7942,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>50.009</v>
+        <v>50.017</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>49.978</v>
+        <v>49.983</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -8024,7 +8024,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>50.021</v>
+        <v>50.008</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -8065,7 +8065,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>85.05</v>
+        <v>85.04600000000001</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -8086,7 +8086,7 @@
         </is>
       </c>
       <c r="I187" t="n">
-        <v>0.02</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="188">
@@ -8106,7 +8106,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>85.033</v>
+        <v>85.036</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -8127,7 +8127,7 @@
         </is>
       </c>
       <c r="I188" t="n">
-        <v>0.003</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="189">
@@ -8147,7 +8147,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>85.03700000000001</v>
+        <v>85.032</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -8168,7 +8168,7 @@
         </is>
       </c>
       <c r="I189" t="n">
-        <v>0.007</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="190">
@@ -8188,7 +8188,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>85.042</v>
+        <v>85.036</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -8209,7 +8209,7 @@
         </is>
       </c>
       <c r="I190" t="n">
-        <v>0.012</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="191">
@@ -8270,7 +8270,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>85.036</v>
+        <v>85.035</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
         </is>
       </c>
       <c r="I192" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="193">
@@ -8311,7 +8311,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>85.038</v>
+        <v>85.035</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -8332,7 +8332,7 @@
         </is>
       </c>
       <c r="I193" t="n">
-        <v>0.008</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="194">
@@ -8352,7 +8352,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>85.054</v>
+        <v>85.029</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -8369,11 +8369,11 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I194" t="n">
-        <v>0.024</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195">
@@ -8393,7 +8393,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>85.035</v>
+        <v>85.03</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -8410,11 +8410,11 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I195" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196">
@@ -8434,7 +8434,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>85.03700000000001</v>
+        <v>85.024</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -8451,11 +8451,11 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I196" t="n">
-        <v>0.007</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197">
@@ -8475,7 +8475,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>85.04300000000001</v>
+        <v>85.04900000000001</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -8496,7 +8496,7 @@
         </is>
       </c>
       <c r="I197" t="n">
-        <v>0.013</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="198">
@@ -8516,7 +8516,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>85.044</v>
+        <v>85.02500000000001</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -8533,11 +8533,11 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I198" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199">
@@ -8557,7 +8557,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>85.044</v>
+        <v>85.029</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -8574,11 +8574,11 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I199" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200">
@@ -8598,7 +8598,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>85.04000000000001</v>
+        <v>85.029</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -8615,11 +8615,11 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I200" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="201">
@@ -8639,7 +8639,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>85.026</v>
+        <v>85.042</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -8656,11 +8656,11 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>conforming</t>
+          <t>nonconforming</t>
         </is>
       </c>
       <c r="I201" t="n">
-        <v>0</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="202">
@@ -8680,7 +8680,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>12.49</v>
+        <v>12.512</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -8721,7 +8721,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>12.509</v>
+        <v>12.501</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -8762,7 +8762,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>12.49</v>
+        <v>12.523</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -8803,7 +8803,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>12.498</v>
+        <v>12.504</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -8844,7 +8844,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>12.506</v>
+        <v>12.502</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -8885,7 +8885,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>12.49</v>
+        <v>12.497</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -8967,7 +8967,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>12.487</v>
+        <v>12.498</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -9008,7 +9008,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>12.494</v>
+        <v>12.507</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -9049,7 +9049,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>12.503</v>
+        <v>12.51</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>12.484</v>
+        <v>12.492</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -9131,7 +9131,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>12.504</v>
+        <v>12.487</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -9172,7 +9172,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>12.5</v>
+        <v>12.482</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -9213,7 +9213,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>12.506</v>
+        <v>12.505</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -9254,7 +9254,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>12.502</v>
+        <v>12.489</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -9295,7 +9295,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>49.999</v>
+        <v>49.998</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -9336,7 +9336,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>50.006</v>
+        <v>49.988</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -9377,7 +9377,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>50.001</v>
+        <v>49.982</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -9459,7 +9459,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>49.991</v>
+        <v>50.008</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -9500,7 +9500,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>50.002</v>
+        <v>49.994</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -9541,7 +9541,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>49.986</v>
+        <v>49.974</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -9582,7 +9582,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>49.999</v>
+        <v>49.995</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -9623,7 +9623,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>49.991</v>
+        <v>50.004</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -9664,7 +9664,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>49.993</v>
+        <v>49.985</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -9705,7 +9705,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>50.012</v>
+        <v>50.002</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -9746,7 +9746,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>50.011</v>
+        <v>50</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -9828,7 +9828,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>49.989</v>
+        <v>50.001</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -9869,7 +9869,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>49.997</v>
+        <v>49.99</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -9910,7 +9910,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>85.002</v>
+        <v>84.98699999999999</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -9951,7 +9951,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>84.996</v>
+        <v>84.976</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -9992,7 +9992,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>84.99299999999999</v>
+        <v>85.02500000000001</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -10033,7 +10033,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>84.996</v>
+        <v>84.98699999999999</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -10074,7 +10074,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>84.995</v>
+        <v>84.997</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -10115,7 +10115,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>85.002</v>
+        <v>84.997</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -10156,7 +10156,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>85.002</v>
+        <v>85.004</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>85</v>
+        <v>85.01000000000001</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -10238,7 +10238,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>85.005</v>
+        <v>85.01000000000001</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -10279,7 +10279,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>85.014</v>
+        <v>84.99299999999999</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -10320,7 +10320,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>85.011</v>
+        <v>84.998</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -10361,7 +10361,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>84.982</v>
+        <v>85.003</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -10402,7 +10402,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>84.96899999999999</v>
+        <v>84.997</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -10419,11 +10419,11 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>nonconforming</t>
+          <t>conforming</t>
         </is>
       </c>
       <c r="I244" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245">
@@ -10443,7 +10443,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>85.011</v>
+        <v>85.01900000000001</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>84.98399999999999</v>
+        <v>85.006</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>12.497</v>
+        <v>12.507</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -10566,7 +10566,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>12.516</v>
+        <v>12.509</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -10607,7 +10607,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>12.507</v>
+        <v>12.493</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -10648,7 +10648,7 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>12.505</v>
+        <v>12.49</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -10689,7 +10689,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>12.526</v>
+        <v>12.5</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -10730,7 +10730,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>12.492</v>
+        <v>12.498</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>12.511</v>
+        <v>12.495</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -10812,7 +10812,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>12.501</v>
+        <v>12.508</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -10853,7 +10853,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>12.503</v>
+        <v>12.511</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>12.518</v>
+        <v>12.501</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -10935,7 +10935,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>12.506</v>
+        <v>12.518</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -10976,7 +10976,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>12.506</v>
+        <v>12.486</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -11017,7 +11017,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>12.513</v>
+        <v>12.498</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -11058,7 +11058,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>12.496</v>
+        <v>12.491</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -11099,7 +11099,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>12.49</v>
+        <v>12.478</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>50.003</v>
+        <v>50.006</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -11181,7 +11181,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>50.011</v>
+        <v>50</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -11222,7 +11222,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>49.983</v>
+        <v>49.981</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -11263,7 +11263,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>49.979</v>
+        <v>50.014</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -11304,7 +11304,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>49.982</v>
+        <v>49.991</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -11345,7 +11345,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>50.015</v>
+        <v>49.99</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -11386,7 +11386,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>49.993</v>
+        <v>50.002</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -11427,7 +11427,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>50.031</v>
+        <v>50.014</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -11468,7 +11468,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>49.993</v>
+        <v>49.988</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>50.002</v>
+        <v>50.001</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -11550,7 +11550,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>50.019</v>
+        <v>50.005</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -11591,7 +11591,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>50.024</v>
+        <v>50.008</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -11632,7 +11632,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>50.025</v>
+        <v>50.002</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -11673,7 +11673,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>50.015</v>
+        <v>49.996</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -11714,7 +11714,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>50.012</v>
+        <v>49.99</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -11755,7 +11755,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>84.997</v>
+        <v>85.03100000000001</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -11772,11 +11772,11 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>conforming</t>
+          <t>nonconforming</t>
         </is>
       </c>
       <c r="I277" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="278">
@@ -11796,7 +11796,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>85</v>
+        <v>85.00700000000001</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -11837,7 +11837,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>84.991</v>
+        <v>85.004</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>84.971</v>
+        <v>85.002</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -11919,7 +11919,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>85.011</v>
+        <v>84.996</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -11960,7 +11960,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>85.009</v>
+        <v>85.004</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -12001,7 +12001,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>84.997</v>
+        <v>84.996</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -12042,7 +12042,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>85.001</v>
+        <v>85.002</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -12083,7 +12083,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>85.006</v>
+        <v>85.01600000000001</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -12124,7 +12124,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>84.98099999999999</v>
+        <v>84.988</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -12165,7 +12165,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>84.994</v>
+        <v>85.014</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -12206,7 +12206,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>85.01000000000001</v>
+        <v>85.01600000000001</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -12247,7 +12247,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>84.985</v>
+        <v>84.999</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -12288,7 +12288,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>85.004</v>
+        <v>84.97499999999999</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -12329,7 +12329,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>84.98399999999999</v>
+        <v>84.99299999999999</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -12370,7 +12370,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>12.496</v>
+        <v>12.489</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -12411,7 +12411,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>12.495</v>
+        <v>12.513</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -12452,7 +12452,7 @@
         </is>
       </c>
       <c r="D294" t="n">
-        <v>12.489</v>
+        <v>12.494</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -12493,7 +12493,7 @@
         </is>
       </c>
       <c r="D295" t="n">
-        <v>12.505</v>
+        <v>12.51</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -12534,7 +12534,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>12.525</v>
+        <v>12.504</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -12575,7 +12575,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>12.487</v>
+        <v>12.522</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -12616,7 +12616,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>12.5</v>
+        <v>12.497</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -12657,7 +12657,7 @@
         </is>
       </c>
       <c r="D299" t="n">
-        <v>12.517</v>
+        <v>12.496</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -12698,7 +12698,7 @@
         </is>
       </c>
       <c r="D300" t="n">
-        <v>12.499</v>
+        <v>12.5</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -12739,7 +12739,7 @@
         </is>
       </c>
       <c r="D301" t="n">
-        <v>12.505</v>
+        <v>12.496</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -12780,7 +12780,7 @@
         </is>
       </c>
       <c r="D302" t="n">
-        <v>12.487</v>
+        <v>12.51</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -12821,7 +12821,7 @@
         </is>
       </c>
       <c r="D303" t="n">
-        <v>12.505</v>
+        <v>12.481</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -12862,7 +12862,7 @@
         </is>
       </c>
       <c r="D304" t="n">
-        <v>12.498</v>
+        <v>12.487</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -12903,7 +12903,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>12.512</v>
+        <v>12.487</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -12944,7 +12944,7 @@
         </is>
       </c>
       <c r="D306" t="n">
-        <v>12.514</v>
+        <v>12.511</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -12985,7 +12985,7 @@
         </is>
       </c>
       <c r="D307" t="n">
-        <v>49.995</v>
+        <v>50</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -13026,7 +13026,7 @@
         </is>
       </c>
       <c r="D308" t="n">
-        <v>50.011</v>
+        <v>50.015</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -13067,7 +13067,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>50.009</v>
+        <v>50.01</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -13108,7 +13108,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>50.004</v>
+        <v>50.011</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -13149,7 +13149,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>50.024</v>
+        <v>50.012</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -13190,7 +13190,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>50.022</v>
+        <v>50.016</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -13231,7 +13231,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>50.03</v>
+        <v>50.022</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -13272,7 +13272,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>50.037</v>
+        <v>50.036</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -13313,7 +13313,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>50.041</v>
+        <v>50.043</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -13354,7 +13354,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>50.049</v>
+        <v>50.037</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -13395,7 +13395,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>50.048</v>
+        <v>50.054</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -13412,11 +13412,11 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>conforming</t>
+          <t>nonconforming</t>
         </is>
       </c>
       <c r="I317" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="318">
@@ -13436,7 +13436,7 @@
         </is>
       </c>
       <c r="D318" t="n">
-        <v>50.058</v>
+        <v>50.053</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -13457,7 +13457,7 @@
         </is>
       </c>
       <c r="I318" t="n">
-        <v>0.008</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="319">
@@ -13477,7 +13477,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>50.059</v>
+        <v>50.061</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -13498,7 +13498,7 @@
         </is>
       </c>
       <c r="I319" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="320">
@@ -13518,7 +13518,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>50.069</v>
+        <v>50.073</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -13539,7 +13539,7 @@
         </is>
       </c>
       <c r="I320" t="n">
-        <v>0.019</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="321">
@@ -13559,7 +13559,7 @@
         </is>
       </c>
       <c r="D321" t="n">
-        <v>50.073</v>
+        <v>50.074</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -13580,7 +13580,7 @@
         </is>
       </c>
       <c r="I321" t="n">
-        <v>0.023</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="322">
@@ -13600,7 +13600,7 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>85.001</v>
+        <v>84.998</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -13641,7 +13641,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>84.98</v>
+        <v>85.006</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -13682,7 +13682,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>84.996</v>
+        <v>84.97799999999999</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -13723,7 +13723,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>84.989</v>
+        <v>84.98399999999999</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -13764,7 +13764,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>85.004</v>
+        <v>84.983</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -13805,7 +13805,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>85.01900000000001</v>
+        <v>85.002</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -13846,7 +13846,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>84.974</v>
+        <v>85.024</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -13887,7 +13887,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>85.002</v>
+        <v>85.03100000000001</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -13904,11 +13904,11 @@
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>conforming</t>
+          <t>nonconforming</t>
         </is>
       </c>
       <c r="I329" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="330">
@@ -13928,7 +13928,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>84.998</v>
+        <v>85.009</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -13969,7 +13969,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>85.009</v>
+        <v>85.00700000000001</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -14010,7 +14010,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>85.003</v>
+        <v>84.97499999999999</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -14051,7 +14051,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>84.989</v>
+        <v>84.992</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -14092,7 +14092,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>84.996</v>
+        <v>84.989</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -14133,7 +14133,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>84.989</v>
+        <v>84.991</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -14174,7 +14174,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>85.015</v>
+        <v>84.998</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -14215,7 +14215,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>12.503</v>
+        <v>12.504</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -14256,7 +14256,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>12.498</v>
+        <v>12.513</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -14297,7 +14297,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>12.51</v>
+        <v>12.5</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -14338,7 +14338,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>12.51</v>
+        <v>12.489</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -14379,7 +14379,7 @@
         </is>
       </c>
       <c r="D341" t="n">
-        <v>12.479</v>
+        <v>12.498</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -14420,7 +14420,7 @@
         </is>
       </c>
       <c r="D342" t="n">
-        <v>12.516</v>
+        <v>12.491</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -14461,7 +14461,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>12.48</v>
+        <v>12.492</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -14502,7 +14502,7 @@
         </is>
       </c>
       <c r="D344" t="n">
-        <v>12.512</v>
+        <v>12.498</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -14543,7 +14543,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>12.514</v>
+        <v>12.49</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -14584,7 +14584,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>12.487</v>
+        <v>12.496</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -14625,7 +14625,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>12.495</v>
+        <v>12.477</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -14666,7 +14666,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>12.487</v>
+        <v>12.503</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -14707,7 +14707,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>12.497</v>
+        <v>12.5</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -14748,7 +14748,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>12.496</v>
+        <v>12.49</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -14789,7 +14789,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>12.509</v>
+        <v>12.508</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>50.032</v>
+        <v>50.011</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -14871,7 +14871,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>49.982</v>
+        <v>50.012</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -14912,7 +14912,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>50.003</v>
+        <v>50.015</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -14953,7 +14953,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>50.006</v>
+        <v>50.001</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -14994,7 +14994,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>50.013</v>
+        <v>50.002</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -15035,7 +15035,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>50.001</v>
+        <v>49.993</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -15076,7 +15076,7 @@
         </is>
       </c>
       <c r="D358" t="n">
-        <v>50.004</v>
+        <v>49.996</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -15117,7 +15117,7 @@
         </is>
       </c>
       <c r="D359" t="n">
-        <v>49.995</v>
+        <v>50.007</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -15158,7 +15158,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>50.003</v>
+        <v>50.014</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -15199,7 +15199,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>49.996</v>
+        <v>49.998</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -15240,7 +15240,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>50.007</v>
+        <v>49.995</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -15281,7 +15281,7 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>49.996</v>
+        <v>50</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -15322,7 +15322,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>50.005</v>
+        <v>50.007</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -15363,7 +15363,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>50</v>
+        <v>49.983</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -15404,7 +15404,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>50.014</v>
+        <v>49.972</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>

</xml_diff>